<commit_message>
Add bonus experiments and re-measure AMP dtype throughput
Bonus (RUBRIC section 2), none of which uses fold-0 test:
- final config F01 on folds 1 and 2 (seed 0), test once per fold
- DINOv2 ViT-S/14 frozen linear probe vs DeiT-S IN-1k (same protocol)
- distribution shift on val (dark/blur/noise) with ECE before/after TS
- test-time adaptation: BN-adapt (B05, B06) and Tent (F01)
- Grad-CAM and attention rollout for Chinee apple <-> Snake weed errors
- ONNX export (static batch 1) and latency vs PyTorch

Also replace the untraceable AMP dtype numbers with a logged benchmark,
add unit tests for the bonus helpers, and update report, README,
notebook and results.xlsx (new Bonus_* and AMP_dtype sheets).
</commit_message>
<xml_diff>
--- a/submissions/2A202602515_DoanDuyBach/results.xlsx
+++ b/submissions/2A202602515_DoanDuyBach/results.xlsx
@@ -15,6 +15,13 @@
     <sheet name="PerClass" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Latency" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Decomposition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="AMP_dtype" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Bonus_Folds" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Bonus_Probe" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Bonus_Shift" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Bonus_TTA" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Bonus_Attention" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Bonus_ONNX" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1081,6 +1088,2472 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>exp_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>fold</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>seed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>số ảnh test</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>T (khớp trên val của fold)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 val</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 test</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>top-1 test</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ECE test</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>recall Chinee Apple test</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>recall Snake Weed test</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>3507</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0.6386907814438205</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0.9618191875705855</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.9651368222876372</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0.9734816082121471</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>0.008143472244083204</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>0.9469026548672567</v>
+      </c>
+      <c r="K2" s="5" t="n">
+        <v>0.9411764705882353</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F01_fold1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>3503</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.6352442768268319</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.9616127358520724</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.9523652461522892</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0.9651727091064801</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0.01192633729374826</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>0.9333333333333333</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0.812807881773399</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>F01_fold2</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>3501</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0.6222150535862662</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0.9692312613965177</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0.9627703709178951</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>0.971151099685804</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.009648278109111697</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>0.9288888888888889</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.916256157635468</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mean ± std qua 3 fold</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tổng hợp</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.6321 ± 0.0087</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.9642 ± 0.0043</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.9601 ± 0.0068</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0.9699 ± 0.0043</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0.0099 ± 0.0019</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0.9364 ± 0.0094</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0.8901 ± 0.0681</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>mô hình</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>timm</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>cách dùng</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>#tham số (M)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>C (CV 5-fold trên train)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 val</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>top-1 val</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ECE val</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>F1 Chinee Apple val</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>F1 Snake Weed val</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DINOv2 ViT-S/14 (tự giám sát LVD-142M), đóng băng + hồi quy logistic</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vit_small_patch14_dinov2.lvd142m</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>linear probe (đặc trưng đóng băng)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>22.056192</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0.9074542106357332</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.9251642387889174</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0.01532566704875365</v>
+      </c>
+      <c r="I2" s="5" t="n">
+        <v>0.8681818181818182</v>
+      </c>
+      <c r="J2" s="5" t="n">
+        <v>0.8564231738035264</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DeiT-S (có giám sát ImageNet-1k), đóng băng + hồi quy logistic (cùng giao thức)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>deit_small_patch16_224.fb_in1k</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>linear probe (đặc trưng đóng băng)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>21.665664</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.8332183870562708</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.8694658668951728</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0.02693442813466867</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0.7470449172576832</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>0.755784061696658</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>T01: DeiT-S đóng băng, head train 10 epoch có augmentation (Bước 2)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>tham chiếu</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="5" t="n">
+        <v>0.7328850613040376</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.7932019423021994</v>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" s="5" t="n">
+        <v>0.6261682242990654</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0.6537396121883656</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>B03: DeiT-S tinh chỉnh toàn bộ (Bước 1)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>tham chiếu</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="5" t="n">
+        <v>0.9507544566343044</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.9642959154527277</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" s="5" t="n">
+        <v>0.8944954128440367</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0.896551724137931</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>B02: ConvNeXt-T tinh chỉnh toàn bộ (Bước 1)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>tham chiếu</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="4" t="n">
+        <v>0.968785755586721</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>0.9765781205369894</v>
+      </c>
+      <c r="H6" s="3" t="inlineStr"/>
+      <c r="I6" s="4" t="n">
+        <v>0.9517241379310346</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>0.9268292682926828</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>B01: ResNet-50 tinh chỉnh toàn bộ (Bước 1)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>tham chiếu</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" s="5" t="n">
+        <v>0.7772771770370791</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.8369037417880606</v>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" s="5" t="n">
+        <v>0.6379310344827587</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>0.6891191709844561</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>B06: MobileNetV3 tinh chỉnh toàn bộ (Bước 1)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>tham chiếu</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" s="5" t="n">
+        <v>0.7049573327705817</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.7857754927163667</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" s="5" t="n">
+        <v>0.7029702970297029</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>0.7304785894206548</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="33" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>cấu hình</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>suy luận</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>điều kiện (val)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>số seed</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 val</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>std macro-F1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>top-1 val</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>F1 Chinee Apple</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>F1 Snake Weed</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ECE (T = 1)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>ECE (T khớp val sạch)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ECE (T oracle, khớp lại trên ảnh lệch)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>T oracle</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>độ tin cậy TB (T khớp val sạch)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>sạch</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>0.9666494132850995</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>0.004331606674393049</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0.9754355898314767</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>0.9329549659131939</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.9239260445813202</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.08378873841309892</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0.006206628294412588</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>0.006206628294412588</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>0.6206652944259926</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>0.9801106070642258</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,5</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.9315764828784792</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.01013867473982087</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.9460154241645244</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0.8853853648328069</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>0.8666536473682124</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>0.09125296382344765</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0.01416602290950162</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>0.009346642022822689</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>0.6609483027779811</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0.9590815546983187</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,3</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>0.8832935688361032</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0.02038642605682617</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.9021232028944112</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0.829037295852193</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>0.8430150011609627</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0.07460906940248081</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0.03974565113531631</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>0.01927274450256401</v>
+      </c>
+      <c r="M4" s="5" t="n">
+        <v>0.7352168828912372</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0.9414331992604174</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mờ σ = 1,5 px</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0.6673838269202564</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.006040311298146181</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.768351899457298</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0.5553732419746433</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>0.4148155816127433</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0.07192765945591556</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0.1605225632559515</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>0.07271702321177104</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>0.9908582635253268</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0.9282407096261345</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>mờ σ = 3 px</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0.2936812001909775</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0.03433051799488054</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0.5925925925925926</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0.4289531337598358</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>0.1669686435469179</v>
+      </c>
+      <c r="J6" s="5" t="n">
+        <v>0.1672690493582496</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0.3108780784826248</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>0.1015467603087358</v>
+      </c>
+      <c r="M6" s="5" t="n">
+        <v>1.246029642065688</v>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0.9032228379570242</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,05</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.9527755999546209</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.003004849710670121</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.9655336570503664</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.9135210521904371</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>0.9117249485747868</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>0.08516049838828955</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0.009690238274823381</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>0.009237534432221504</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>0.6373803687838026</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0.9745147125684365</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ảnh đầy đủ 288</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,10</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.8832865587762392</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.01631290619473129</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.916214414929068</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0.8336670258172317</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>0.8701552618884807</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>0.07459187122750034</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0.03525932751969519</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>0.01984234237112777</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>0.7205647815566794</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0.94970874765853</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>sạch</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.9522278693421221</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.005316043203616738</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.9657240788346186</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0.8942963750760827</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0.9082653801073485</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>0.007978776261602904</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0.006501352887470383</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0.006501352887470383</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>1.069948607386992</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0.9640325165074652</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,5</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0.9225728953208737</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0.005525272862882938</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0.9414453013424735</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0.8641659657627851</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>0.8495048974691813</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>0.01374733172740808</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0.01021513276081269</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>0.009223665428826675</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>1.098609047417391</v>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>0.9439670314017364</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,3</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.8637662646891151</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.02284647967352618</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.8846043987432163</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.8267858013618651</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0.8090188517566409</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>0.03419753705371496</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.02723812620366619</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>0.01318025497599457</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>1.214314308116254</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0.9079507140947861</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>mờ σ = 1,5 px</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0.5603394118899591</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0.03364763568741704</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0.7061791868989813</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0.5418430793131565</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>0.4018221743305999</v>
+      </c>
+      <c r="J12" s="5" t="n">
+        <v>0.215166603423537</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0.2082029463503291</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>0.08878629714158</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>2.05708788676337</v>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>0.9143404607672078</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>mờ σ = 3 px</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.2714742868425677</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.03219541385059719</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.5805008092925831</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0.3844930424249837</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0.1218763787912999</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>0.312822618000774</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0.2999667987205319</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>0.08636426991850177</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>2.165755817897649</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0.8800763521745557</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,05</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0.935436043695808</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0.005762367846402784</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0.9536322955346092</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>0.8709638647756144</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>0.8909259259259259</v>
+      </c>
+      <c r="J14" s="5" t="n">
+        <v>0.01094447165694183</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>0.008828481190451674</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>0.00837576278025484</v>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>1.098641794268475</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>0.9554743303198737</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>CenterCrop 224</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,10</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.8698689621364509</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.009122740252821605</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.9037417880605542</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0.8192985257917607</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0.8520771153184983</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>0.03118085937541693</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0.02536444889909302</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0.01248908989875618</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>1.228747586884373</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0.9255728701173062</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>phương pháp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>mô hình</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>điều kiện (val)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 trước</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 precise-BN (train sạch)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 sau</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>ECE trước</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ECE sau</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>sạch</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0.7660887520222311</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0.8640412992407709</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0.8661382103189867</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>0.03605225413001041</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0.0233298439476732</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,5</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>0.6630509915182247</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.6291002577970031</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.8634675965799486</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0.08146658488086057</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0.02488569976346011</v>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,3</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>0.3703866644874095</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>0.2756481611078233</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>0.8620699968074103</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0.1699114766095219</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>0.02521201971741702</v>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mờ σ = 1,5 px</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>0.2818523159596629</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>0.18524279621221</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>0.7903585899754739</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0.2337990196859578</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>0.05005402748138205</v>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>mờ σ = 3 px</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0.1048096339151151</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>0.09681418889124188</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0.5780480784789369</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0.1948839718698718</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>0.1334179703671808</v>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,05</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0.1283627503206206</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>0.5244850318563452</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.8516888996842044</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0.268625287181372</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>0.02581578374282181</v>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B05</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,10</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0.07327301065217043</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0.08233191236506869</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0.8014154036747164</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0.1974344307162788</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>0.04696142360932846</v>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>sạch</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0.7068366842251657</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.8758277665639715</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.8746189481546258</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.02628664092438807</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0.01300948774374079</v>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,5</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0.69163066306725</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>0.6565299440918332</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0.8743728110323764</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0.03678290048341552</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>0.01624347759691047</v>
+      </c>
+      <c r="I10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,3</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0.2963862700289382</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.2500080185644991</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.8741781277799707</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.1168589133779608</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.01936265236165821</v>
+      </c>
+      <c r="I11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>mờ σ = 1,5 px</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0.2936935097521954</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>0.1866048316918061</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0.8067673930639674</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0.2538958349309647</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>0.02482903448377403</v>
+      </c>
+      <c r="I12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>mờ σ = 3 px</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0.08409761458111882</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.08669919424224015</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.5858258359684777</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.5147553010332551</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0.1157586672183368</v>
+      </c>
+      <c r="I13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,05</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0.1096637236366241</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>0.645100468198615</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0.8683494722763401</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0.401854822378486</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>0.01316051297349022</v>
+      </c>
+      <c r="I14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BN-adapt: thống kê BN tính lại trên chính ảnh lệch (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,10</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0.1213961336071648</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.118993679145641</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.8403215522817472</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.2144237650791287</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0.01987160584384856</v>
+      </c>
+      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tent: cập nhật γ/β LayerNorm, cực tiểu entropy, online 1 lượt (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>F01 seed 0</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,5</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0.9391936600724464</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" s="5" t="n">
+        <v>0.944434123957439</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0.009295444492168027</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>0.008265658220989267</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>ECE với T khớp trên val sạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tent: cập nhật γ/β LayerNorm, cực tiểu entropy, online 1 lượt (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>F01 seed 0</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>thiếu sáng ×0,3</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0.895451771415956</v>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" s="5" t="n">
+        <v>0.9124948909318271</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.03068524766525118</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0.02436845478267612</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>ECE với T khớp trên val sạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tent: cập nhật γ/β LayerNorm, cực tiểu entropy, online 1 lượt (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>F01 seed 0</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>mờ σ = 1,5 px</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0.6737007240710957</v>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" s="5" t="n">
+        <v>0.6582598745631962</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0.1620529200485235</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>0.1724765688661341</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ECE với T khớp trên val sạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tent: cập nhật γ/β LayerNorm, cực tiểu entropy, online 1 lượt (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>F01 seed 0</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>mờ σ = 3 px</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0.2653128823208873</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" s="5" t="n">
+        <v>0.2524708982070519</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0.3446406072483196</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0.3623795172914778</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>ECE với T khớp trên val sạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tent: cập nhật γ/β LayerNorm, cực tiểu entropy, online 1 lượt (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>F01 seed 0</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,05</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0.9501854337238341</v>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" s="5" t="n">
+        <v>0.9497603360085736</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0.01074184014225434</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>0.01162745301486685</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>ECE với T khớp trên val sạch</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tent: cập nhật γ/β LayerNorm, cực tiểu entropy, online 1 lượt (không nhãn)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>F01 seed 0</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>nhiễu σ = 0,10</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0.8938874463410037</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" s="5" t="n">
+        <v>0.8975669961519908</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0.03362035958014909</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.03373346095340077</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>ECE với T khớp trên val sạch</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>nhóm ảnh val (Chinee apple + Snake weed)</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>số ảnh</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>diện tích thực vật xanh (ExG-Otsu)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Grad-CAM: tập trung vào thực vật (tỉ số)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Grad-CAM: entropy chuẩn hoá</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Grad-CAM: std entropy</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>rollout: tập trung vào thực vật (tỉ số)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>rollout: entropy chuẩn hoá</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>đoán sai</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>34</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>0.387673327432825</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1.065546247113907</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>0.8389072466399718</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>0.1216887750634521</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>1.053158426250269</v>
+      </c>
+      <c r="H2" s="5" t="n">
+        <v>0.9935263147359386</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>đoán đúng</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>394</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>0.5065306431444664</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>1.083050579322496</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>0.8837521269462418</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>0.06550821319656137</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1.020433229074143</v>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>0.9939788273783553</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>backend</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dtype</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>độ phân giải</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>p50 (ms)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p95 (ms)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>p99 (ms)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>số lần đo</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>warmup</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>macro-F1 val</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>sai khác logit lớn nhất so với PyTorch CPU</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>tỉ lệ trùng nhãn đoán</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>PyTorch, GPU (MPS)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>288</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>11.55814549974821</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>14.65561839972906</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>14.93286740960684</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>0.9618191875705855</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>1.358985900878906e-05</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PyTorch, CPU</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>288</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>24.35131250013001</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>27.30644585035407</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>28.71917249934996</v>
+      </c>
+      <c r="H3" t="n">
+        <v>100</v>
+      </c>
+      <c r="I3" t="n">
+        <v>10</v>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>0.9618191875705855</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ONNX Runtime, CPU</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>288</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>30.93720800006849</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>33.14642289988114</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>35.05858791948413</v>
+      </c>
+      <c r="H4" t="n">
+        <v>100</v>
+      </c>
+      <c r="I4" t="n">
+        <v>10</v>
+      </c>
+      <c r="J4" s="5" t="n">
+        <v>0.9618191875705855</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>1.609325408935547e-05</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ONNX Runtime, CoreML EP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>288</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>11.871874499775</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>12.30761280030492</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>12.85943750006482</v>
+      </c>
+      <c r="H5" t="n">
+        <v>100</v>
+      </c>
+      <c r="I5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0.9618191875705855</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>1.817941665649414e-05</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6654,4 +9127,172 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>mô hình</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>thiết bị</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dtype</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>độ phân giải</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tốc độ train (ảnh/s)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>thời gian một bước (ms)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>torch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>fp32</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>64</v>
+      </c>
+      <c r="E2" t="n">
+        <v>224</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>44.58316122138962</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>1435.519560449984</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2.14.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>fp16</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>64</v>
+      </c>
+      <c r="E3" t="n">
+        <v>224</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>60.86368734399919</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>1051.530112499995</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2.14.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>resnet50</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>mps</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bf16</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>64</v>
+      </c>
+      <c r="E4" t="n">
+        <v>224</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>58.44481019759617</v>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>1095.050181250008</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2.14.1</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>